<commit_message>
[feat] Penalty 테이블에 HeroSkillName 필드 추가
- Penalty.xlsx에 HeroSkillName 컬럼 추가
- JSON 재생성 및 업로드
- GameData.cs에 HeroSkillName 필드 반영
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Penalty.xlsx
+++ b/JsonConverter/ExcelFiles/Penalty.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GameProjects\ACE\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D795792-775E-4617-9CD7-220D5060B07F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F466FAD3-62D0-4775-8AE5-54A2A40FE379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25710" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-16130" yWindow="1900" windowWidth="20870" windowHeight="11880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Penalty" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="82">
   <si>
     <t>string</t>
   </si>
@@ -259,6 +259,41 @@
   <si>
     <t>변신 중 힘 딸려서 근력 저하</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>유발 스킬 이름</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>TriggerSkillName</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>뱃살튕기기</t>
+  </si>
+  <si>
+    <t>라떼는말이야</t>
+  </si>
+  <si>
+    <t>럭키방패</t>
+  </si>
+  <si>
+    <t>오십견킥</t>
+  </si>
+  <si>
+    <t>감으로쏘기</t>
+  </si>
+  <si>
+    <t>힘껏노려보기</t>
+  </si>
+  <si>
+    <t>망치날라가유</t>
+  </si>
+  <si>
+    <t>뿌리감기</t>
+  </si>
+  <si>
+    <t>아몬드가죽으면</t>
   </si>
 </sst>
 </file>
@@ -660,22 +695,23 @@
   <sheetPr codeName="Sheet1">
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:S1000"/>
+  <dimension ref="A1:T1000"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="11.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.5703125" style="2" customWidth="1"/>
-    <col min="3" max="4" width="24.7109375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="18.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.28515625" style="2" customWidth="1"/>
-    <col min="9" max="9" width="48.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="26.5703125" style="2" customWidth="1"/>
-    <col min="11" max="16384" width="12.5703125" style="2"/>
+    <col min="3" max="3" width="24.7109375" style="2" customWidth="1"/>
+    <col min="4" max="5" width="19.28515625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="18.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.28515625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="48.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="26.5703125" style="2" customWidth="1"/>
+    <col min="12" max="16384" width="12.5703125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="13" customFormat="1" ht="15.75" customHeight="1">
+    <row r="1" spans="1:20" s="13" customFormat="1" ht="15.75" customHeight="1">
       <c r="A1" s="12" t="s">
         <v>2</v>
       </c>
@@ -689,22 +725,25 @@
         <v>16</v>
       </c>
       <c r="E1" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="G1" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="H1" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="I1" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="J1" s="12" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:19" s="13" customFormat="1" ht="12.75">
+    <row r="2" spans="1:20" s="13" customFormat="1" ht="12.75">
       <c r="A2" s="12" t="s">
         <v>1</v>
       </c>
@@ -718,23 +757,26 @@
         <v>1</v>
       </c>
       <c r="E2" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="G2" s="12" t="s">
         <v>1</v>
-      </c>
-      <c r="G2" s="12" t="s">
-        <v>24</v>
       </c>
       <c r="H2" s="12" t="s">
         <v>24</v>
       </c>
       <c r="I2" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="J2" s="12"/>
-    </row>
-    <row r="3" spans="1:19" s="15" customFormat="1" ht="15.75" customHeight="1">
+      <c r="K2" s="12"/>
+    </row>
+    <row r="3" spans="1:20" s="15" customFormat="1" ht="15.75" customHeight="1">
       <c r="A3" s="14" t="s">
         <v>7</v>
       </c>
@@ -748,22 +790,25 @@
         <v>10</v>
       </c>
       <c r="E3" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="F3" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="G3" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="14" t="s">
+      <c r="H3" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="14" t="s">
+      <c r="I3" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="I3" s="14" t="s">
+      <c r="J3" s="14" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="15.75" customHeight="1">
+    <row r="4" spans="1:20" ht="15.75" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
@@ -776,23 +821,25 @@
       <c r="D4" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="F4" s="3">
         <v>2</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G4" s="3">
+      <c r="H4" s="3">
         <v>10</v>
       </c>
-      <c r="H4" s="3">
+      <c r="I4" s="3">
         <v>2</v>
       </c>
-      <c r="I4" s="11" t="s">
+      <c r="J4" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="J4" s="10"/>
-      <c r="K4" s="4"/>
+      <c r="K4" s="10"/>
       <c r="L4" s="4"/>
       <c r="M4" s="4"/>
       <c r="N4" s="4"/>
@@ -801,8 +848,9 @@
       <c r="Q4" s="4"/>
       <c r="R4" s="4"/>
       <c r="S4" s="4"/>
-    </row>
-    <row r="5" spans="1:19" ht="15.75" customHeight="1">
+      <c r="T4" s="4"/>
+    </row>
+    <row r="5" spans="1:20" ht="15.75" customHeight="1">
       <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
@@ -815,22 +863,24 @@
       <c r="D5" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F5" s="3">
         <v>2</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="G5" s="3">
+      <c r="H5" s="3">
         <v>10</v>
       </c>
-      <c r="H5" s="3">
+      <c r="I5" s="3">
         <v>2</v>
       </c>
-      <c r="I5" s="11" t="s">
+      <c r="J5" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="J5" s="4"/>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
       <c r="M5" s="4"/>
@@ -840,8 +890,9 @@
       <c r="Q5" s="4"/>
       <c r="R5" s="4"/>
       <c r="S5" s="4"/>
-    </row>
-    <row r="6" spans="1:19" ht="15.75" customHeight="1">
+      <c r="T5" s="4"/>
+    </row>
+    <row r="6" spans="1:20" ht="15.75" customHeight="1">
       <c r="A6" s="3" t="s">
         <v>25</v>
       </c>
@@ -854,22 +905,24 @@
       <c r="D6" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="F6" s="3">
         <v>2</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="G6" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="G6" s="3">
+      <c r="H6" s="3">
         <v>10</v>
       </c>
-      <c r="H6" s="3">
+      <c r="I6" s="3">
         <v>2</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="J6" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="J6" s="4"/>
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
       <c r="M6" s="4"/>
@@ -879,8 +932,9 @@
       <c r="Q6" s="4"/>
       <c r="R6" s="4"/>
       <c r="S6" s="4"/>
-    </row>
-    <row r="7" spans="1:19" ht="15.75" customHeight="1">
+      <c r="T6" s="4"/>
+    </row>
+    <row r="7" spans="1:20" ht="15.75" customHeight="1">
       <c r="A7" s="3" t="s">
         <v>26</v>
       </c>
@@ -893,22 +947,24 @@
       <c r="D7" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F7" s="3">
         <v>2</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="G7" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="G7" s="3">
+      <c r="H7" s="3">
         <v>10</v>
       </c>
-      <c r="H7" s="3">
+      <c r="I7" s="3">
         <v>2</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="J7" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="J7" s="4"/>
       <c r="K7" s="4"/>
       <c r="L7" s="4"/>
       <c r="M7" s="4"/>
@@ -918,8 +974,9 @@
       <c r="Q7" s="4"/>
       <c r="R7" s="4"/>
       <c r="S7" s="4"/>
-    </row>
-    <row r="8" spans="1:19" ht="15.75" customHeight="1">
+      <c r="T7" s="4"/>
+    </row>
+    <row r="8" spans="1:20" ht="15.75" customHeight="1">
       <c r="A8" s="3" t="s">
         <v>27</v>
       </c>
@@ -932,22 +989,24 @@
       <c r="D8" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="F8" s="3">
         <v>2</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="G8" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="3">
+      <c r="H8" s="3">
         <v>10</v>
       </c>
-      <c r="H8" s="3">
+      <c r="I8" s="3">
         <v>2</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="J8" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="J8" s="4"/>
       <c r="K8" s="4"/>
       <c r="L8" s="4"/>
       <c r="M8" s="4"/>
@@ -957,8 +1016,9 @@
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
-    </row>
-    <row r="9" spans="1:19" ht="15.75" customHeight="1">
+      <c r="T8" s="4"/>
+    </row>
+    <row r="9" spans="1:20" ht="15.75" customHeight="1">
       <c r="A9" s="3" t="s">
         <v>28</v>
       </c>
@@ -971,22 +1031,24 @@
       <c r="D9" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F9" s="3">
         <v>2</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="G9" s="3">
+      <c r="H9" s="3">
         <v>10</v>
       </c>
-      <c r="H9" s="3">
+      <c r="I9" s="3">
         <v>2</v>
       </c>
-      <c r="I9" s="3" t="s">
+      <c r="J9" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="J9" s="4"/>
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
       <c r="M9" s="4"/>
@@ -996,8 +1058,9 @@
       <c r="Q9" s="4"/>
       <c r="R9" s="4"/>
       <c r="S9" s="4"/>
-    </row>
-    <row r="10" spans="1:19" ht="15.75" customHeight="1">
+      <c r="T9" s="4"/>
+    </row>
+    <row r="10" spans="1:20" ht="15.75" customHeight="1">
       <c r="A10" s="3" t="s">
         <v>29</v>
       </c>
@@ -1010,22 +1073,24 @@
       <c r="D10" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E10" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="F10" s="3">
         <v>2</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="G10" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="3">
+      <c r="H10" s="3">
         <v>10</v>
       </c>
-      <c r="H10" s="3">
+      <c r="I10" s="3">
         <v>2</v>
       </c>
-      <c r="I10" s="3" t="s">
+      <c r="J10" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="J10" s="4"/>
       <c r="K10" s="4"/>
       <c r="L10" s="4"/>
       <c r="M10" s="4"/>
@@ -1035,8 +1100,9 @@
       <c r="Q10" s="4"/>
       <c r="R10" s="4"/>
       <c r="S10" s="4"/>
-    </row>
-    <row r="11" spans="1:19" ht="15.75" customHeight="1">
+      <c r="T10" s="4"/>
+    </row>
+    <row r="11" spans="1:20" ht="15.75" customHeight="1">
       <c r="A11" s="3" t="s">
         <v>30</v>
       </c>
@@ -1049,22 +1115,24 @@
       <c r="D11" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F11" s="1">
         <v>2</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G11" s="1">
+      <c r="H11" s="1">
         <v>10</v>
       </c>
-      <c r="H11" s="1">
+      <c r="I11" s="1">
         <v>2</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="J11" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="J11" s="4"/>
       <c r="K11" s="4"/>
       <c r="L11" s="4"/>
       <c r="M11" s="4"/>
@@ -1074,8 +1142,9 @@
       <c r="Q11" s="4"/>
       <c r="R11" s="4"/>
       <c r="S11" s="4"/>
-    </row>
-    <row r="12" spans="1:19" ht="15.75" customHeight="1">
+      <c r="T11" s="4"/>
+    </row>
+    <row r="12" spans="1:20" ht="15.75" customHeight="1">
       <c r="A12" s="3" t="s">
         <v>31</v>
       </c>
@@ -1088,22 +1157,24 @@
       <c r="D12" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="F12" s="5">
         <v>2</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="G12" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G12" s="5">
+      <c r="H12" s="5">
         <v>10</v>
       </c>
-      <c r="H12" s="5">
+      <c r="I12" s="5">
         <v>2</v>
       </c>
-      <c r="I12" s="5" t="s">
+      <c r="J12" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="J12" s="4"/>
       <c r="K12" s="4"/>
       <c r="L12" s="4"/>
       <c r="M12" s="4"/>
@@ -1113,8 +1184,9 @@
       <c r="Q12" s="4"/>
       <c r="R12" s="4"/>
       <c r="S12" s="4"/>
-    </row>
-    <row r="13" spans="1:19" ht="15.75" customHeight="1">
+      <c r="T12" s="4"/>
+    </row>
+    <row r="13" spans="1:20" ht="15.75" customHeight="1">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -1124,7 +1196,7 @@
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
-      <c r="J13" s="4"/>
+      <c r="J13" s="3"/>
       <c r="K13" s="4"/>
       <c r="L13" s="4"/>
       <c r="M13" s="4"/>
@@ -1134,8 +1206,9 @@
       <c r="Q13" s="4"/>
       <c r="R13" s="4"/>
       <c r="S13" s="4"/>
-    </row>
-    <row r="14" spans="1:19" ht="15.75" customHeight="1">
+      <c r="T13" s="4"/>
+    </row>
+    <row r="14" spans="1:20" ht="15.75" customHeight="1">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -1145,7 +1218,7 @@
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
-      <c r="J14" s="4"/>
+      <c r="J14" s="1"/>
       <c r="K14" s="4"/>
       <c r="L14" s="4"/>
       <c r="M14" s="4"/>
@@ -1155,8 +1228,9 @@
       <c r="Q14" s="4"/>
       <c r="R14" s="4"/>
       <c r="S14" s="4"/>
-    </row>
-    <row r="15" spans="1:19" ht="15.75" customHeight="1">
+      <c r="T14" s="4"/>
+    </row>
+    <row r="15" spans="1:20" ht="15.75" customHeight="1">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -1166,7 +1240,7 @@
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
-      <c r="J15" s="4"/>
+      <c r="J15" s="1"/>
       <c r="K15" s="4"/>
       <c r="L15" s="4"/>
       <c r="M15" s="4"/>
@@ -1176,8 +1250,9 @@
       <c r="Q15" s="4"/>
       <c r="R15" s="4"/>
       <c r="S15" s="4"/>
-    </row>
-    <row r="16" spans="1:19" ht="15.75" customHeight="1">
+      <c r="T15" s="4"/>
+    </row>
+    <row r="16" spans="1:20" ht="15.75" customHeight="1">
       <c r="A16" s="6"/>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
@@ -1187,8 +1262,9 @@
       <c r="G16" s="7"/>
       <c r="H16" s="7"/>
       <c r="I16" s="7"/>
-    </row>
-    <row r="17" spans="1:9" ht="15.75" customHeight="1">
+      <c r="J16" s="7"/>
+    </row>
+    <row r="17" spans="1:10" ht="15.75" customHeight="1">
       <c r="A17" s="7"/>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -1198,8 +1274,9 @@
       <c r="G17" s="7"/>
       <c r="H17" s="7"/>
       <c r="I17" s="7"/>
-    </row>
-    <row r="18" spans="1:9" ht="15.75" customHeight="1">
+      <c r="J17" s="7"/>
+    </row>
+    <row r="18" spans="1:10" ht="15.75" customHeight="1">
       <c r="A18" s="7"/>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
@@ -1209,8 +1286,9 @@
       <c r="G18" s="7"/>
       <c r="H18" s="7"/>
       <c r="I18" s="7"/>
-    </row>
-    <row r="19" spans="1:9" ht="15.75" customHeight="1">
+      <c r="J18" s="7"/>
+    </row>
+    <row r="19" spans="1:10" ht="15.75" customHeight="1">
       <c r="A19" s="7"/>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -1220,8 +1298,9 @@
       <c r="G19" s="7"/>
       <c r="H19" s="7"/>
       <c r="I19" s="7"/>
-    </row>
-    <row r="20" spans="1:9" ht="15.75" customHeight="1">
+      <c r="J19" s="7"/>
+    </row>
+    <row r="20" spans="1:10" ht="15.75" customHeight="1">
       <c r="A20" s="7"/>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -1231,8 +1310,9 @@
       <c r="G20" s="7"/>
       <c r="H20" s="7"/>
       <c r="I20" s="7"/>
-    </row>
-    <row r="21" spans="1:9" ht="15.75" customHeight="1">
+      <c r="J20" s="7"/>
+    </row>
+    <row r="21" spans="1:10" ht="15.75" customHeight="1">
       <c r="A21" s="7"/>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
@@ -1242,8 +1322,9 @@
       <c r="G21" s="7"/>
       <c r="H21" s="7"/>
       <c r="I21" s="7"/>
-    </row>
-    <row r="22" spans="1:9" ht="15.75" customHeight="1">
+      <c r="J21" s="7"/>
+    </row>
+    <row r="22" spans="1:10" ht="15.75" customHeight="1">
       <c r="A22" s="7"/>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
@@ -1253,8 +1334,9 @@
       <c r="G22" s="7"/>
       <c r="H22" s="7"/>
       <c r="I22" s="7"/>
-    </row>
-    <row r="23" spans="1:9" ht="15.75" customHeight="1">
+      <c r="J22" s="7"/>
+    </row>
+    <row r="23" spans="1:10" ht="15.75" customHeight="1">
       <c r="A23" s="7"/>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
@@ -1264,8 +1346,9 @@
       <c r="G23" s="7"/>
       <c r="H23" s="7"/>
       <c r="I23" s="7"/>
-    </row>
-    <row r="24" spans="1:9" ht="15.75" customHeight="1">
+      <c r="J23" s="7"/>
+    </row>
+    <row r="24" spans="1:10" ht="15.75" customHeight="1">
       <c r="A24" s="7"/>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
@@ -1275,8 +1358,9 @@
       <c r="G24" s="7"/>
       <c r="H24" s="7"/>
       <c r="I24" s="7"/>
-    </row>
-    <row r="25" spans="1:9" ht="15.75" customHeight="1">
+      <c r="J24" s="7"/>
+    </row>
+    <row r="25" spans="1:10" ht="15.75" customHeight="1">
       <c r="A25" s="7"/>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
@@ -1286,8 +1370,9 @@
       <c r="G25" s="7"/>
       <c r="H25" s="7"/>
       <c r="I25" s="7"/>
-    </row>
-    <row r="26" spans="1:9" ht="15.75" customHeight="1">
+      <c r="J25" s="7"/>
+    </row>
+    <row r="26" spans="1:10" ht="15.75" customHeight="1">
       <c r="A26" s="8"/>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
@@ -1297,8 +1382,9 @@
       <c r="G26" s="8"/>
       <c r="H26" s="8"/>
       <c r="I26" s="8"/>
-    </row>
-    <row r="27" spans="1:9" ht="15.75" customHeight="1">
+      <c r="J26" s="8"/>
+    </row>
+    <row r="27" spans="1:10" ht="15.75" customHeight="1">
       <c r="A27" s="8"/>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
@@ -1308,8 +1394,9 @@
       <c r="G27" s="8"/>
       <c r="H27" s="8"/>
       <c r="I27" s="8"/>
-    </row>
-    <row r="28" spans="1:9" ht="15.75" customHeight="1">
+      <c r="J27" s="8"/>
+    </row>
+    <row r="28" spans="1:10" ht="15.75" customHeight="1">
       <c r="A28" s="8"/>
       <c r="B28" s="8"/>
       <c r="C28" s="8"/>
@@ -1319,8 +1406,9 @@
       <c r="G28" s="8"/>
       <c r="H28" s="8"/>
       <c r="I28" s="8"/>
-    </row>
-    <row r="29" spans="1:9" ht="15.75" customHeight="1">
+      <c r="J28" s="8"/>
+    </row>
+    <row r="29" spans="1:10" ht="15.75" customHeight="1">
       <c r="A29" s="8"/>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
@@ -1330,8 +1418,9 @@
       <c r="G29" s="8"/>
       <c r="H29" s="8"/>
       <c r="I29" s="8"/>
-    </row>
-    <row r="30" spans="1:9" ht="15.75" customHeight="1">
+      <c r="J29" s="8"/>
+    </row>
+    <row r="30" spans="1:10" ht="15.75" customHeight="1">
       <c r="A30" s="8"/>
       <c r="B30" s="8"/>
       <c r="C30" s="8"/>
@@ -1341,8 +1430,9 @@
       <c r="G30" s="8"/>
       <c r="H30" s="8"/>
       <c r="I30" s="8"/>
-    </row>
-    <row r="31" spans="1:9" ht="15.75" customHeight="1">
+      <c r="J30" s="8"/>
+    </row>
+    <row r="31" spans="1:10" ht="15.75" customHeight="1">
       <c r="A31" s="8"/>
       <c r="B31" s="8"/>
       <c r="C31" s="8"/>
@@ -1352,8 +1442,9 @@
       <c r="G31" s="8"/>
       <c r="H31" s="8"/>
       <c r="I31" s="8"/>
-    </row>
-    <row r="32" spans="1:9" ht="15.75" customHeight="1">
+      <c r="J31" s="8"/>
+    </row>
+    <row r="32" spans="1:10" ht="15.75" customHeight="1">
       <c r="A32" s="9"/>
       <c r="B32" s="9"/>
       <c r="C32" s="9"/>
@@ -1363,8 +1454,9 @@
       <c r="G32" s="9"/>
       <c r="H32" s="9"/>
       <c r="I32" s="9"/>
-    </row>
-    <row r="33" spans="1:9" ht="15.75" customHeight="1">
+      <c r="J32" s="9"/>
+    </row>
+    <row r="33" spans="1:10" ht="15.75" customHeight="1">
       <c r="A33" s="9"/>
       <c r="B33" s="9"/>
       <c r="C33" s="9"/>
@@ -1374,8 +1466,9 @@
       <c r="G33" s="9"/>
       <c r="H33" s="9"/>
       <c r="I33" s="9"/>
-    </row>
-    <row r="34" spans="1:9" ht="15.75" customHeight="1">
+      <c r="J33" s="9"/>
+    </row>
+    <row r="34" spans="1:10" ht="15.75" customHeight="1">
       <c r="A34" s="9"/>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
@@ -1385,8 +1478,9 @@
       <c r="G34" s="9"/>
       <c r="H34" s="9"/>
       <c r="I34" s="9"/>
-    </row>
-    <row r="35" spans="1:9" ht="15.75" customHeight="1">
+      <c r="J34" s="9"/>
+    </row>
+    <row r="35" spans="1:10" ht="15.75" customHeight="1">
       <c r="A35" s="9"/>
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
@@ -1396,20 +1490,21 @@
       <c r="G35" s="9"/>
       <c r="H35" s="9"/>
       <c r="I35" s="9"/>
-    </row>
-    <row r="36" spans="1:9" ht="15.75" customHeight="1"/>
-    <row r="37" spans="1:9" ht="15.75" customHeight="1"/>
-    <row r="38" spans="1:9" ht="15.75" customHeight="1"/>
-    <row r="39" spans="1:9" ht="15.75" customHeight="1"/>
-    <row r="40" spans="1:9" ht="15.75" customHeight="1"/>
-    <row r="41" spans="1:9" ht="15.75" customHeight="1"/>
-    <row r="42" spans="1:9" ht="15.75" customHeight="1"/>
-    <row r="43" spans="1:9" ht="15.75" customHeight="1"/>
-    <row r="44" spans="1:9" ht="15.75" customHeight="1"/>
-    <row r="45" spans="1:9" ht="15.75" customHeight="1"/>
-    <row r="46" spans="1:9" ht="15.75" customHeight="1"/>
-    <row r="47" spans="1:9" ht="15.75" customHeight="1"/>
-    <row r="48" spans="1:9" ht="15.75" customHeight="1"/>
+      <c r="J35" s="9"/>
+    </row>
+    <row r="36" spans="1:10" ht="15.75" customHeight="1"/>
+    <row r="37" spans="1:10" ht="15.75" customHeight="1"/>
+    <row r="38" spans="1:10" ht="15.75" customHeight="1"/>
+    <row r="39" spans="1:10" ht="15.75" customHeight="1"/>
+    <row r="40" spans="1:10" ht="15.75" customHeight="1"/>
+    <row r="41" spans="1:10" ht="15.75" customHeight="1"/>
+    <row r="42" spans="1:10" ht="15.75" customHeight="1"/>
+    <row r="43" spans="1:10" ht="15.75" customHeight="1"/>
+    <row r="44" spans="1:10" ht="15.75" customHeight="1"/>
+    <row r="45" spans="1:10" ht="15.75" customHeight="1"/>
+    <row r="46" spans="1:10" ht="15.75" customHeight="1"/>
+    <row r="47" spans="1:10" ht="15.75" customHeight="1"/>
+    <row r="48" spans="1:10" ht="15.75" customHeight="1"/>
     <row r="49" ht="15.75" customHeight="1"/>
     <row r="50" ht="15.75" customHeight="1"/>
     <row r="51" ht="15.75" customHeight="1"/>

</xml_diff>